<commit_message>
Changes in testng.xml file
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\KshitijRajuGanare\IdeaProjects\Selenium_Framework_OrangeHRMRef\src\test\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hp\IdeaProjects\Selenium_Framework_OrangeHRM\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8268BB3C-F993-4920-ABF3-0A830717DE19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB10BE78-FC8D-48DF-9D5E-3BB9307F9C53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="26">
   <si>
     <t>UserRole</t>
   </si>
@@ -54,9 +54,6 @@
     <t>ESS</t>
   </si>
   <si>
-    <t>Disabled</t>
-  </si>
-  <si>
     <t>Ranga_Billa_01</t>
   </si>
   <si>
@@ -93,60 +90,6 @@
     <t>Admin_Access1</t>
   </si>
   <si>
-    <t>Ian_Inactive</t>
-  </si>
-  <si>
-    <t>Log_Off_99</t>
-  </si>
-  <si>
-    <t>Jasmine_Flow</t>
-  </si>
-  <si>
-    <t>Flow_Test_1</t>
-  </si>
-  <si>
-    <t>Kev_Automation</t>
-  </si>
-  <si>
-    <t>Selenium_#1</t>
-  </si>
-  <si>
-    <t>Laura_Dev_Test</t>
-  </si>
-  <si>
-    <t>Quality_1st</t>
-  </si>
-  <si>
-    <t>Mike_Security</t>
-  </si>
-  <si>
-    <t>Shield_990</t>
-  </si>
-  <si>
-    <t>Nina_Verify</t>
-  </si>
-  <si>
-    <t>Check_Pass_2</t>
-  </si>
-  <si>
-    <t>Oscar_Wild_02</t>
-  </si>
-  <si>
-    <t>Wild_Card_5</t>
-  </si>
-  <si>
-    <t>Paula_Manager</t>
-  </si>
-  <si>
-    <t>Lead_Mngr_0</t>
-  </si>
-  <si>
-    <t>Quentin_QA</t>
-  </si>
-  <si>
-    <t>QA_Expert_!</t>
-  </si>
-  <si>
     <t>Test@12346</t>
   </si>
   <si>
@@ -159,28 +102,7 @@
     <t>Admin_Access2</t>
   </si>
   <si>
-    <t>Log_Off_100</t>
-  </si>
-  <si>
-    <t>Flow_Test_2</t>
-  </si>
-  <si>
-    <t>Selenium_#2</t>
-  </si>
-  <si>
-    <t>Shield_991</t>
-  </si>
-  <si>
-    <t>Check_Pass_3</t>
-  </si>
-  <si>
-    <t>Wild_Card_6</t>
-  </si>
-  <si>
-    <t>Lead_Mngr_1</t>
-  </si>
-  <si>
-    <t>John</t>
+    <t>Johna</t>
   </si>
 </sst>
 </file>
@@ -223,7 +145,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -246,11 +168,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
@@ -258,10 +195,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
   </cellXfs>
@@ -547,29 +487,29 @@
   <dimension ref="A1:F16"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9.36328125" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.6328125" style="2" customWidth="1"/>
+    <col min="1" max="1" width="13.26953125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="17.54296875" style="2" customWidth="1"/>
     <col min="3" max="3" width="14.90625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="15.7265625" style="2" customWidth="1"/>
-    <col min="5" max="5" width="16.26953125" style="2" customWidth="1"/>
-    <col min="6" max="6" width="15.90625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="18.81640625" style="2" customWidth="1"/>
+    <col min="5" max="5" width="18" style="2" customWidth="1"/>
+    <col min="6" max="6" width="20" style="2" customWidth="1"/>
     <col min="7" max="16384" width="8.7265625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:6" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
@@ -577,304 +517,196 @@
       </c>
     </row>
     <row r="2" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="C2" s="4" t="s">
+      <c r="B2" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="F2" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="4" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="4" t="s">
+      <c r="E3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="C3" s="4" t="s">
+      <c r="B5" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="E4" s="4" t="s">
+      <c r="D5" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F4" s="4" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="4" t="s">
+      <c r="E5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="C5" s="4" t="s">
+      <c r="B6" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="E5" s="4" t="s">
+      <c r="D6" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="F5" s="4" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D6" s="4" t="s">
+      <c r="E6" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E6" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="F6" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A7" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="C7" s="4" t="s">
+      <c r="B7" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>7</v>
       </c>
       <c r="D7" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E7" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E7" s="4" t="s">
-        <v>21</v>
-      </c>
       <c r="F7" s="4" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D9" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="E9" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A10" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A11" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="F11" s="4" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A12" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="F12" s="4" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A13" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="E13" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="F13" s="4" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A14" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="E14" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="F14" s="4" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A15" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="E15" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="F15" s="4" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A16" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D16" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="E16" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="F16" s="4" t="s">
-        <v>39</v>
-      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A8" s="5"/>
+      <c r="B8" s="5"/>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
+      <c r="F8" s="5"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A9" s="5"/>
+      <c r="B9" s="5"/>
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
+      <c r="F9" s="5"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A10" s="5"/>
+      <c r="B10" s="5"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A11" s="5"/>
+      <c r="B11" s="5"/>
+      <c r="C11" s="5"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A12" s="5"/>
+      <c r="B12" s="5"/>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+      <c r="F12" s="5"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A13" s="5"/>
+      <c r="B13" s="5"/>
+      <c r="C13" s="5"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+      <c r="F13" s="5"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A14" s="5"/>
+      <c r="B14" s="5"/>
+      <c r="C14" s="5"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
+      <c r="F14" s="5"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A15" s="5"/>
+      <c r="B15" s="5"/>
+      <c r="C15" s="5"/>
+      <c r="D15" s="5"/>
+      <c r="E15" s="5"/>
+      <c r="F15" s="5"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A16" s="5"/>
+      <c r="B16" s="5"/>
+      <c r="C16" s="5"/>
+      <c r="D16" s="5"/>
+      <c r="E16" s="5"/>
+      <c r="F16" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>